<commit_message>
WIP with a working test
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Tests/Resources/ConfidenceReport.xlsx
+++ b/GenBOE/GenBOE.Tests/Resources/ConfidenceReport.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26731"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{088FC061-8586-4FE7-AB9A-8807A3A3493E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6B90B4-3CBA-4537-9961-19D2EDC94E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1725" yWindow="-13875" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CLINs" sheetId="1" r:id="rId1"/>
@@ -18,36 +18,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Do not change the genBOE CLIN IDs. 
-The genBOE CLIN IDs in column A are unique identifiers for CLINs. One will be automatically generated for each new CLIN once the import is complete. 
-By default, this column is hidden to prevent accidental edits. </t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>genBOE CLIN ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>ContractTypes</t>
   </si>
@@ -71,7 +43,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,12 +64,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -166,7 +132,7 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -471,22 +437,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.140625" style="4" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="40.5703125" style="3" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="56.28515625" style="3" customWidth="1"/>
     <col min="6" max="6" width="58.28515625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:6" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
@@ -500,11 +467,8 @@
       <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="3" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -512,7 +476,6 @@
     <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -526,7 +489,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -540,16 +503,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -656,27 +615,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E141511F-2C2D-45F4-A120-F9C297666AB6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -701,9 +655,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E141511F-2C2D-45F4-A120-F9C297666AB6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated template, updated tests and code based on MR feedback
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Tests/Resources/ConfidenceReport.xlsx
+++ b/GenBOE/GenBOE.Tests/Resources/ConfidenceReport.xlsx
@@ -3,15 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26731"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6B90B4-3CBA-4537-9961-19D2EDC94E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{673B041D-C873-4DB0-9B37-67F895E96C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3870" yWindow="4215" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="CLINs" sheetId="1" r:id="rId1"/>
+    <sheet name="Confidence Report" sheetId="1" r:id="rId1"/>
     <sheet name="Options Lists" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Confidence Report'!$A$2:$E$2</definedName>
     <definedName name="ContractTypes">'Options Lists'!$A$2</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
@@ -470,6 +471,7 @@
     </row>
     <row r="3" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
+  <autoFilter ref="A2:E2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>

</xml_diff>